<commit_message>
Update $0-$300 payout model with real data from 1,686 tournaments
- Replaced estimated payouts with real scraped data ($201-$300 range)
- 1st: $5,500 -> $7,594, 10th+: $500 -> $813 (richer than estimated)
- Average field 420 players, avg pool $95K
- New "Outgrown Current Level" classification for players profitable higher
- Becker flips from losing to +$44 at $300
- All cleaned transcripts (46 files) from 3 parallel batch agents
- Updated leak analysis and bulk analysis with real payout data
- Redeployed to poker.alphabreak.vip

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/stake_move_analysis.xlsx
+++ b/stake_move_analysis.xlsx
@@ -722,13 +722,13 @@
         <v>0.0825</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>89</v>
+        <v>268</v>
       </c>
       <c r="I2" s="5" t="n">
-        <v>35.4</v>
+        <v>100.1</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0.206</v>
@@ -790,7 +790,7 @@
       </c>
       <c r="AC2" s="7" t="inlineStr">
         <is>
-          <t>Hourly jumps 3048% ($14 -&gt; $429/hr). Profitable at all steps.</t>
+          <t>Hourly jumps 939% ($41 -&gt; $429/hr). Profitable at all steps.</t>
         </is>
       </c>
     </row>
@@ -823,13 +823,13 @@
         <v>0.0477</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>-57</v>
+        <v>44</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>-22.7</v>
+        <v>16.3</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>-9</v>
+        <v>7</v>
       </c>
       <c r="K3" s="3" t="n">
         <v>0.122</v>
@@ -891,7 +891,7 @@
       </c>
       <c r="AC3" s="7" t="inlineStr">
         <is>
-          <t>Breakeven/losing at $300 ($-57) but payout structure at $301-$600 is profitable ($+646/entry, $99/hr).</t>
+          <t>Hourly jumps 1383% ($7 -&gt; $99/hr). Profitable at all steps.</t>
         </is>
       </c>
     </row>
@@ -924,13 +924,13 @@
         <v>0.1455</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>271</v>
+        <v>559</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>108.4</v>
+        <v>208.7</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>42</v>
+        <v>86</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0.3129</v>
@@ -992,7 +992,7 @@
       </c>
       <c r="AC4" s="7" t="inlineStr">
         <is>
-          <t>Hourly jumps 3272% ($42 -&gt; $1,405/hr). Profitable at all steps.</t>
+          <t>Hourly jumps 1534% ($86 -&gt; $1,405/hr). Profitable at all steps.</t>
         </is>
       </c>
     </row>
@@ -1025,13 +1025,13 @@
         <v>0.1079</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>203</v>
+        <v>448</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>81</v>
+        <v>167.1</v>
       </c>
       <c r="J5" s="4" t="n">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>0.3055</v>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="AC5" s="7" t="inlineStr">
         <is>
-          <t>Hourly jumps 3322% ($31 -&gt; $1,066/hr). Profitable at all steps.</t>
+          <t>Hourly jumps 1448% ($69 -&gt; $1,066/hr). Profitable at all steps.</t>
         </is>
       </c>
     </row>
@@ -1126,13 +1126,13 @@
         <v>0.0835</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>113</v>
+        <v>313</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>45.2</v>
+        <v>116.7</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0.2864</v>
@@ -1194,7 +1194,7 @@
       </c>
       <c r="AC6" s="7" t="inlineStr">
         <is>
-          <t>Hourly jumps 2611% ($17 -&gt; $471/hr). Profitable at all steps.</t>
+          <t>Hourly jumps 879% ($48 -&gt; $471/hr). Profitable at all steps.</t>
         </is>
       </c>
     </row>
@@ -1227,13 +1227,13 @@
         <v>0.0209</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>-89</v>
+        <v>-8</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>-35.6</v>
+        <v>-2.9</v>
       </c>
       <c r="J7" s="4" t="n">
-        <v>-14</v>
+        <v>-1</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>0.1541</v>
@@ -1282,11 +1282,11 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>$301-$600</t>
+          <t>$0-$300</t>
         </is>
       </c>
       <c r="AA7" s="4" t="n">
-        <v>-8</v>
+        <v>-1</v>
       </c>
       <c r="AB7" s="8" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="AC7" s="7" t="inlineStr">
         <is>
-          <t>Losing at current level ($-89/entry) and no higher tier is profitable.</t>
+          <t>Losing at current level ($-8/entry) and no higher tier is profitable.</t>
         </is>
       </c>
     </row>
@@ -1328,13 +1328,13 @@
         <v>0.0373</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>-119</v>
+        <v>-49</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>-47.5</v>
+        <v>-18.3</v>
       </c>
       <c r="J8" s="4" t="n">
-        <v>-18</v>
+        <v>-8</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0.0694</v>
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="AA8" s="4" t="n">
-        <v>-18</v>
+        <v>-8</v>
       </c>
       <c r="AB8" s="8" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="AC8" s="7" t="inlineStr">
         <is>
-          <t>Losing at current level ($-119/entry) and no higher tier is profitable.</t>
+          <t>Losing at current level ($-49/entry) and no higher tier is profitable.</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>5500</v>
+        <v>7594</v>
       </c>
       <c r="C2" s="10" t="n">
         <v>52077</v>
@@ -1485,7 +1485,7 @@
         <v>172903</v>
       </c>
       <c r="F2" s="11" t="n">
-        <v>9.5</v>
+        <v>6.9</v>
       </c>
       <c r="G2" s="11" t="n">
         <v>1.8</v>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>3500</v>
+        <v>5843</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>40797</v>
@@ -1513,7 +1513,7 @@
         <v>127200</v>
       </c>
       <c r="F3" s="11" t="n">
-        <v>11.7</v>
+        <v>7</v>
       </c>
       <c r="G3" s="11" t="n">
         <v>1.7</v>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="B4" s="10" t="n">
-        <v>2400</v>
+        <v>4298</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>29397</v>
@@ -1541,7 +1541,7 @@
         <v>96212</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>12.2</v>
+        <v>6.8</v>
       </c>
       <c r="G4" s="11" t="n">
         <v>1.8</v>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="B5" s="10" t="n">
-        <v>1100</v>
+        <v>2051</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>12331</v>
@@ -1569,7 +1569,7 @@
         <v>38937</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>11.2</v>
+        <v>6</v>
       </c>
       <c r="G5" s="11" t="n">
         <v>1.7</v>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>500</v>
+        <v>813</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>1924</v>
@@ -1597,7 +1597,7 @@
         <v>5697</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3.8</v>
+        <v>2.4</v>
       </c>
       <c r="G6" s="11" t="n">
         <v>1.9</v>
@@ -1613,7 +1613,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>596</v>
@@ -1625,7 +1625,7 @@
         <v>1783</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>2.4</v>
+        <v>2.2</v>
       </c>
       <c r="G7" s="12" t="n">
         <v>1.7</v>
@@ -1641,7 +1641,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>25000</v>
+        <v>26800</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>59600</v>
@@ -1662,10 +1662,8 @@
           <t>Sample size</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>est</t>
-        </is>
+      <c r="B9" s="9" t="n">
+        <v>1686</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>130</v>

</xml_diff>